<commit_message>
Set PD LTSF bids to break-even CPC; add broad-campaign manual build sheet
Auto bulk files (US, CA) rebuilt with close-match at each product's PD
break-even CPC. Broad campaigns get a manual build sheet for the PPC
manager, and the campaign plan reflects the new bid caps.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Wv13KPDszSjtnJt4JhRwx
</commit_message>
<xml_diff>
--- a/PD_LTSF_Auto_Bulk_CA.xlsx
+++ b/PD_LTSF_Auto_Bulk_CA.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>2.02</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="4">
@@ -1104,7 +1104,7 @@
         </is>
       </c>
       <c r="AB11" t="n">
-        <v>2.02</v>
+        <v>1.4</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="AB12" t="n">
-        <v>1.82</v>
+        <v>1.26</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="AB13" t="n">
-        <v>1.62</v>
+        <v>1.12</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
@@ -1230,7 +1230,7 @@
         </is>
       </c>
       <c r="AB14" t="n">
-        <v>1.21</v>
+        <v>0.84</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>2.02</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="17">
@@ -1564,7 +1564,7 @@
         </is>
       </c>
       <c r="AB22" t="n">
-        <v>2.02</v>
+        <v>1.3</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="AB23" t="n">
-        <v>1.82</v>
+        <v>1.17</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
@@ -1648,7 +1648,7 @@
         </is>
       </c>
       <c r="AB24" t="n">
-        <v>1.62</v>
+        <v>1.04</v>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="AB25" t="n">
-        <v>1.21</v>
+        <v>0.78</v>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
@@ -1792,7 +1792,7 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>1.17</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="28">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="AB30" t="n">
-        <v>1.17</v>
+        <v>0.7</v>
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="AB31" t="n">
-        <v>1.05</v>
+        <v>0.63</v>
       </c>
       <c r="AJ31" t="inlineStr">
         <is>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="AB32" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ32" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="AB33" t="n">
-        <v>0.7</v>
+        <v>0.42</v>
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="Z35" t="n">
-        <v>1.2</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="36">
@@ -2562,7 +2562,7 @@
         </is>
       </c>
       <c r="AB46" t="n">
-        <v>1.2</v>
+        <v>0.65</v>
       </c>
       <c r="AJ46" t="inlineStr">
         <is>
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="AB47" t="n">
-        <v>1.08</v>
+        <v>0.59</v>
       </c>
       <c r="AJ47" t="inlineStr">
         <is>
@@ -2646,7 +2646,7 @@
         </is>
       </c>
       <c r="AB48" t="n">
-        <v>0.96</v>
+        <v>0.52</v>
       </c>
       <c r="AJ48" t="inlineStr">
         <is>
@@ -2688,7 +2688,7 @@
         </is>
       </c>
       <c r="AB49" t="n">
-        <v>0.72</v>
+        <v>0.39</v>
       </c>
       <c r="AJ49" t="inlineStr">
         <is>

</xml_diff>